<commit_message>
Apply feature mapping to dataset tables and retrain classifiers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/dataset/tables/накладки.xlsx
+++ b/data/dataset/tables/накладки.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="накладки" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="накладки" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'накладки'!$A$1:$H$112</definedName>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.140625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -452,25 +452,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>материал</t>
+          <t>сохранность</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>сохранность</t>
+          <t>форма</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>форма</t>
+          <t>крепление</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>крепление</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>орнамент</t>
         </is>
@@ -492,25 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ажурная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
-        <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -532,25 +522,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ажурная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -572,25 +557,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
-        <is>
-          <t>клепка</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -612,25 +592,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
-        <is>
-          <t>клепка</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -652,25 +627,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
-        <is>
-          <t>клепка</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -692,25 +662,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>дисковидная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -732,25 +697,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>дисковидная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -772,25 +732,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>каплевидная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -812,25 +767,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>каплевидная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -852,25 +802,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>каплевидная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -892,25 +837,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>подовальная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -932,25 +872,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>подовальная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -972,25 +907,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>подовальная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1012,25 +942,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>фигурная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1052,25 +977,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>фигурная</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1092,25 +1012,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1132,25 +1047,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1172,25 +1082,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1212,25 +1117,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1252,25 +1152,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">четырехлепестковая </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -1292,25 +1187,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">четырехлепестковая </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -1332,25 +1222,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1372,25 +1257,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1412,25 +1292,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -1452,12 +1327,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Бронза, олово, медь, и другой металл, камень</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1468,16 +1343,6 @@
       <c r="G26" t="inlineStr">
         <is>
           <t>не указано</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1362,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Цветной металл, пластик. стекло</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>смешанный</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1513,16 +1378,6 @@
       <c r="G27" t="inlineStr">
         <is>
           <t>не указано</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -1542,12 +1397,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Цветной металл, пластик. стекло</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>смешанный</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1558,16 +1413,6 @@
       <c r="G28" t="inlineStr">
         <is>
           <t>не указано</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -1587,25 +1432,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ввиде меча</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1627,25 +1467,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>ввиде меча</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1667,25 +1502,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1707,25 +1537,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1747,25 +1572,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>подпрямоугольная с овальным краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1787,25 +1607,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>подпрямоугольная с овальным краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1827,25 +1642,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">прямоугольная с петелькой </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1867,25 +1677,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">прямоугольная с петелькой </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1907,25 +1712,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">прямоугольная с петелькой </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1947,25 +1747,20 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">прямоугольная с петелькой </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -1987,25 +1782,20 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">прямоугольная с петелькой </t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2027,25 +1817,20 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2067,25 +1852,20 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2107,25 +1887,20 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>трехчастная из полусфер</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2147,25 +1922,20 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>трехчастная из полусфер</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2187,25 +1957,20 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2227,25 +1992,20 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Цветной металл</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2267,25 +2027,20 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>прямоугольная с заоваленными углами</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2307,25 +2062,20 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>прямоугольная с заоваленными углами</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
-        <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -2342,37 +2092,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ворворки</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -2387,37 +2127,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ворворки</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -2432,37 +2162,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ворворки</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -2482,25 +2202,20 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>четырехлепестковая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2522,25 +2237,20 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>четырехлепестковая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2562,25 +2272,20 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>четырехлепестковая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2602,25 +2307,20 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>четырехлепестковая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -2642,32 +2342,22 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -2687,32 +2377,22 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -2732,32 +2412,22 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -2777,32 +2447,22 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -2822,25 +2482,20 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -2862,25 +2517,20 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -2902,25 +2552,20 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -2942,25 +2587,20 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -2982,25 +2622,20 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -3022,25 +2657,20 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -3062,25 +2692,20 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -3102,25 +2727,20 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3142,25 +2762,20 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3182,25 +2797,20 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
-        <is>
-          <t>перемычка</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3222,25 +2832,20 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
-        <is>
-          <t>перемычка</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3262,25 +2867,20 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
-        <is>
-          <t>перемычка</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3302,25 +2902,20 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>фигурная</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>конусовидная</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
-        <is>
-          <t>перемычка</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3342,25 +2937,20 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -3382,25 +2972,20 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -3422,32 +3007,22 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3467,32 +3042,22 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3512,32 +3077,22 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3557,32 +3112,22 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3602,32 +3147,22 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3647,25 +3182,20 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3687,25 +3217,20 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3727,25 +3252,20 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3767,25 +3287,20 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
@@ -3807,32 +3322,22 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3852,32 +3357,22 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3897,32 +3392,22 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3942,32 +3427,22 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -3987,32 +3462,22 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4032,32 +3497,22 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4077,32 +3532,22 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4122,32 +3567,22 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4167,32 +3602,22 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4207,30 +3632,25 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>двухчастная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -4247,30 +3667,25 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>сломан</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>сломан</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>двухчастная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -4292,25 +3707,20 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4332,25 +3742,20 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4372,25 +3777,20 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4412,25 +3812,20 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внешнее</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
-        <is>
-          <t>петелька</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4447,42 +3842,27 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>пуговица</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>УД80</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -4497,42 +3877,27 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>пуговица</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>УД80</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>не нужно</t>
         </is>
       </c>
     </row>
@@ -4552,32 +3917,22 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>на одной из шести</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>УД80</t>
+          <t>да</t>
         </is>
       </c>
     </row>
@@ -4597,32 +3952,22 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>на одной из шести</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>УД80</t>
+          <t>да</t>
         </is>
       </c>
     </row>
@@ -4642,32 +3987,22 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>шпеньки</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>на одной из шести</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>УД80</t>
+          <t>да</t>
         </is>
       </c>
     </row>
@@ -4682,30 +4017,25 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4722,30 +4052,25 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -4767,32 +4092,22 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4812,32 +4127,22 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4857,32 +4162,22 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4902,32 +4197,22 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>прямоугольная</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>круглая с зубчатым краем</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4947,32 +4232,22 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -4992,32 +4267,22 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>округлая</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>круглая</t>
+          <t>внутреннее</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>через отверстия</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
           <t>нет</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>УД80</t>
         </is>
       </c>
     </row>
@@ -5032,30 +4297,25 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>ажурная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -5072,30 +4332,25 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>нашивка</t>
+          <t>накладки</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Бронза</t>
+          <t>целый</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>целый</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>ажурная</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
         <is>
           <t>да</t>
         </is>

</xml_diff>